<commit_message>
Update "Community Roles" "Community Roles.xlsx".
</commit_message>
<xml_diff>
--- a/Community Roles/Community Roles.xlsx
+++ b/Community Roles/Community Roles.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="21"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="22"/>
   </bookViews>
   <sheets>
     <sheet name="011424" sheetId="1" state="visible" r:id="rId1"/>
@@ -27,7 +27,8 @@
     <sheet name="051725" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="052725" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="072325" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Current" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="072525" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Current" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t>Role</t>
   </si>
@@ -320,6 +321,9 @@
   <si>
     <t xml:space="preserve">7 Days to Die</t>
   </si>
+  <si>
+    <t>Ultron</t>
+  </si>
 </sst>
 </file>
 
@@ -359,7 +363,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -368,11 +372,14 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="23">
     <dxf>
       <font>
         <b val="0"/>
@@ -666,6 +673,7 @@
       </font>
       <alignment horizontal="center" indent="0" readingOrder="0" relativeIndent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
     </dxf>
+    <dxf/>
     <dxf/>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1599,6 +1607,73 @@
   <autoFilter ref="A1:BF20"/>
   <tableColumns count="58">
     <tableColumn id="1" name="Role" dataDxfId="21"/>
+    <tableColumn id="2" name="General Server Permissions"/>
+    <tableColumn id="3" name="View Channels"/>
+    <tableColumn id="4" name="Manage Channels"/>
+    <tableColumn id="5" name="Manage Roles"/>
+    <tableColumn id="6" name="Create Expressions"/>
+    <tableColumn id="7" name="Manage Expressions"/>
+    <tableColumn id="8" name="View Audit Log"/>
+    <tableColumn id="9" name="View Server Insights"/>
+    <tableColumn id="10" name="Manage Webhooks"/>
+    <tableColumn id="11" name="Manage Server"/>
+    <tableColumn id="12" name="Membership Permissions"/>
+    <tableColumn id="13" name="Create Invite"/>
+    <tableColumn id="14" name="Change Nickname"/>
+    <tableColumn id="15" name="Manage Nicknames"/>
+    <tableColumn id="16" name="Kick, Approve, and Reject Members"/>
+    <tableColumn id="17" name="Ban Members"/>
+    <tableColumn id="18" name="Timeout Members"/>
+    <tableColumn id="19" name="Text Channel Permissions"/>
+    <tableColumn id="20" name="Send Messages"/>
+    <tableColumn id="21" name="Send Messages in Threads"/>
+    <tableColumn id="22" name="Create Public Threads"/>
+    <tableColumn id="23" name="Create Private Threads"/>
+    <tableColumn id="24" name="Embed Links"/>
+    <tableColumn id="25" name="Attach Files"/>
+    <tableColumn id="26" name="Add Reactions"/>
+    <tableColumn id="27" name="Use External Emoji"/>
+    <tableColumn id="28" name="Use External Stickers"/>
+    <tableColumn id="29" name="Mention @everyone, @here, and All Roles"/>
+    <tableColumn id="30" name="Manage Messages"/>
+    <tableColumn id="31" name="Manage Threads"/>
+    <tableColumn id="32" name="Read Message History"/>
+    <tableColumn id="33" name="Send Text-to-Speech Messages"/>
+    <tableColumn id="34" name="Send Voice Messages"/>
+    <tableColumn id="35" name="Create Polls"/>
+    <tableColumn id="36" name="Voice Channel Permissions"/>
+    <tableColumn id="37" name="Connect"/>
+    <tableColumn id="38" name="Speak"/>
+    <tableColumn id="39" name="Video"/>
+    <tableColumn id="40" name="Use Soundboard"/>
+    <tableColumn id="41" name="Use External Sounds"/>
+    <tableColumn id="42" name="Use Voice Activity"/>
+    <tableColumn id="43" name="Priority Speaker"/>
+    <tableColumn id="44" name="Mute Members"/>
+    <tableColumn id="45" name="Deafen Members"/>
+    <tableColumn id="46" name="Move Members"/>
+    <tableColumn id="47" name="Set Voice Channel Status"/>
+    <tableColumn id="48" name="Apps Permissions"/>
+    <tableColumn id="49" name="Use Application Commands"/>
+    <tableColumn id="50" name="Use Activities"/>
+    <tableColumn id="51" name="Use External Apps"/>
+    <tableColumn id="52" name="Stage Channel Permissions"/>
+    <tableColumn id="53" name="Request to Speak"/>
+    <tableColumn id="54" name="Events Permissions"/>
+    <tableColumn id="55" name="Create Events"/>
+    <tableColumn id="56" name="Manage Events"/>
+    <tableColumn id="57" name="Advanced Permissions"/>
+    <tableColumn id="58" name="Administrator"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleDark1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" displayName="Table18" ref="A1:BF21">
+  <autoFilter ref="A1:BF21"/>
+  <tableColumns count="58">
+    <tableColumn id="1" name="Role" dataDxfId="22"/>
     <tableColumn id="2" name="General Server Permissions"/>
     <tableColumn id="3" name="View Channels"/>
     <tableColumn id="4" name="Manage Channels"/>
@@ -47687,6 +47762,3312 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col bestFit="1" customWidth="1" min="1" max="1" style="2" width="32.375"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" width="33.00390625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" width="18.75390625"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="22.00390625"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" width="18.00390625"/>
+    <col bestFit="1" customWidth="1" min="6" max="6" width="23.75390625"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" width="25.25390625"/>
+    <col bestFit="1" customWidth="1" min="8" max="8" width="19.125"/>
+    <col bestFit="1" customWidth="1" min="9" max="9" width="24.875"/>
+    <col bestFit="1" customWidth="1" min="10" max="10" width="23.375"/>
+    <col bestFit="1" customWidth="1" min="11" max="11" width="18.875"/>
+    <col bestFit="1" customWidth="1" min="12" max="12" width="30.375"/>
+    <col bestFit="1" customWidth="1" min="13" max="13" width="16.25390625"/>
+    <col bestFit="1" customWidth="1" min="14" max="14" width="22.375"/>
+    <col bestFit="1" customWidth="1" min="15" max="15" width="23.875"/>
+    <col bestFit="1" customWidth="1" min="16" max="16" width="41.25390625"/>
+    <col bestFit="1" customWidth="1" min="17" max="17" width="17.75390625"/>
+    <col bestFit="1" customWidth="1" min="18" max="18" width="22.375"/>
+    <col bestFit="1" customWidth="1" min="19" max="19" width="31.00390625"/>
+    <col bestFit="1" customWidth="1" min="20" max="20" width="19.75390625"/>
+    <col bestFit="1" customWidth="1" min="21" max="21" width="31.75390625"/>
+    <col bestFit="1" customWidth="1" min="22" max="22" width="26.50390625"/>
+    <col bestFit="1" customWidth="1" min="23" max="23" width="27.25390625"/>
+    <col bestFit="1" customWidth="1" min="24" max="24" width="16.875"/>
+    <col bestFit="1" customWidth="1" min="25" max="25" width="15.50390625"/>
+    <col bestFit="1" customWidth="1" min="26" max="26" width="18.50390625"/>
+    <col bestFit="1" customWidth="1" min="27" max="27" width="23.25390625"/>
+    <col bestFit="1" customWidth="1" min="28" max="28" width="25.75390625"/>
+    <col bestFit="1" customWidth="1" min="29" max="29" width="48.00390625"/>
+    <col bestFit="1" customWidth="1" min="30" max="30" width="22.75390625"/>
+    <col bestFit="1" customWidth="1" min="31" max="31" width="20.625"/>
+    <col bestFit="1" customWidth="1" min="32" max="32" width="26.875"/>
+    <col bestFit="1" customWidth="1" min="33" max="33" width="36.625"/>
+    <col bestFit="1" customWidth="1" min="34" max="34" width="26.375"/>
+    <col bestFit="1" customWidth="1" min="35" max="35" width="15.75390625"/>
+    <col bestFit="1" customWidth="1" min="36" max="36" width="32.375"/>
+    <col bestFit="1" customWidth="1" min="37" max="37" width="11.75390625"/>
+    <col bestFit="1" customWidth="1" min="38" max="38" width="9.375"/>
+    <col bestFit="1" customWidth="1" min="39" max="39" width="8.875"/>
+    <col bestFit="1" customWidth="1" min="40" max="40" width="20.75390625"/>
+    <col bestFit="1" customWidth="1" min="41" max="41" width="25.25390625"/>
+    <col bestFit="1" customWidth="1" min="42" max="42" width="22.25390625"/>
+    <col bestFit="1" customWidth="1" min="43" max="43" width="20.00390625"/>
+    <col bestFit="1" customWidth="1" min="44" max="44" width="18.875"/>
+    <col bestFit="1" customWidth="1" min="45" max="45" width="21.00390625"/>
+    <col bestFit="1" customWidth="1" min="46" max="46" width="19.375"/>
+    <col bestFit="1" customWidth="1" min="47" max="47" width="29.875"/>
+    <col bestFit="1" customWidth="1" min="48" max="48" width="22.50390625"/>
+    <col bestFit="1" customWidth="1" min="49" max="49" width="32.875"/>
+    <col bestFit="1" customWidth="1" min="50" max="50" width="17.50390625"/>
+    <col bestFit="1" customWidth="1" min="51" max="51" width="22.625"/>
+    <col bestFit="1" customWidth="1" min="52" max="52" width="32.50390625"/>
+    <col bestFit="1" customWidth="1" min="53" max="53" width="21.625"/>
+    <col bestFit="1" customWidth="1" min="54" max="54" width="24.25390625"/>
+    <col bestFit="1" customWidth="1" min="55" max="55" width="17.75390625"/>
+    <col bestFit="1" customWidth="1" min="56" max="56" width="19.25390625"/>
+    <col bestFit="1" customWidth="1" min="57" max="57" width="27.625"/>
+    <col bestFit="1" customWidth="1" min="58" max="58" width="17.625"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="2" customFormat="1" ht="16.5">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AO1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AQ1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AS1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AU1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AV1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AW1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AX1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AY1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AZ1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="BA1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="BB1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="BC1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="BD1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="BE1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="BF1" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" ht="16.5">
+      <c r="A2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K2" t="s">
+        <v>58</v>
+      </c>
+      <c r="M2" t="s">
+        <v>58</v>
+      </c>
+      <c r="N2" t="s">
+        <v>58</v>
+      </c>
+      <c r="O2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>58</v>
+      </c>
+      <c r="R2" t="s">
+        <v>58</v>
+      </c>
+      <c r="T2" t="s">
+        <v>58</v>
+      </c>
+      <c r="U2" t="s">
+        <v>58</v>
+      </c>
+      <c r="V2" t="s">
+        <v>58</v>
+      </c>
+      <c r="W2" t="s">
+        <v>58</v>
+      </c>
+      <c r="X2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>58</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>58</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>58</v>
+      </c>
+      <c r="BF2" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5">
+      <c r="A3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J3" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" t="s">
+        <v>58</v>
+      </c>
+      <c r="N3" t="s">
+        <v>56</v>
+      </c>
+      <c r="O3" t="s">
+        <v>56</v>
+      </c>
+      <c r="P3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>58</v>
+      </c>
+      <c r="R3" t="s">
+        <v>56</v>
+      </c>
+      <c r="T3" t="s">
+        <v>58</v>
+      </c>
+      <c r="U3" t="s">
+        <v>58</v>
+      </c>
+      <c r="V3" t="s">
+        <v>56</v>
+      </c>
+      <c r="W3" t="s">
+        <v>58</v>
+      </c>
+      <c r="X3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AT3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" ht="16.5">
+      <c r="A4" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" t="s">
+        <v>56</v>
+      </c>
+      <c r="J4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K4" t="s">
+        <v>58</v>
+      </c>
+      <c r="M4" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" t="s">
+        <v>58</v>
+      </c>
+      <c r="O4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>58</v>
+      </c>
+      <c r="R4" t="s">
+        <v>56</v>
+      </c>
+      <c r="T4" t="s">
+        <v>58</v>
+      </c>
+      <c r="U4" t="s">
+        <v>56</v>
+      </c>
+      <c r="V4" t="s">
+        <v>56</v>
+      </c>
+      <c r="W4" t="s">
+        <v>56</v>
+      </c>
+      <c r="X4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AT4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AU4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" ht="16.5">
+      <c r="A5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" t="s">
+        <v>56</v>
+      </c>
+      <c r="N5" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5" t="s">
+        <v>56</v>
+      </c>
+      <c r="P5" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>56</v>
+      </c>
+      <c r="R5" t="s">
+        <v>56</v>
+      </c>
+      <c r="T5" t="s">
+        <v>56</v>
+      </c>
+      <c r="U5" t="s">
+        <v>56</v>
+      </c>
+      <c r="V5" t="s">
+        <v>56</v>
+      </c>
+      <c r="W5" t="s">
+        <v>56</v>
+      </c>
+      <c r="X5" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5">
+      <c r="A6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N6" t="s">
+        <v>56</v>
+      </c>
+      <c r="O6" t="s">
+        <v>56</v>
+      </c>
+      <c r="P6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>56</v>
+      </c>
+      <c r="R6" t="s">
+        <v>56</v>
+      </c>
+      <c r="T6" t="s">
+        <v>56</v>
+      </c>
+      <c r="U6" t="s">
+        <v>56</v>
+      </c>
+      <c r="V6" t="s">
+        <v>56</v>
+      </c>
+      <c r="W6" t="s">
+        <v>56</v>
+      </c>
+      <c r="X6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC6" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" ht="16.5">
+      <c r="A7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" t="s">
+        <v>56</v>
+      </c>
+      <c r="N7" t="s">
+        <v>56</v>
+      </c>
+      <c r="O7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P7" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>56</v>
+      </c>
+      <c r="R7" t="s">
+        <v>56</v>
+      </c>
+      <c r="T7" t="s">
+        <v>56</v>
+      </c>
+      <c r="U7" t="s">
+        <v>56</v>
+      </c>
+      <c r="V7" t="s">
+        <v>56</v>
+      </c>
+      <c r="W7" t="s">
+        <v>56</v>
+      </c>
+      <c r="X7" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY7" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA7" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC7" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD7" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5">
+      <c r="A8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" t="s">
+        <v>58</v>
+      </c>
+      <c r="J8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K8" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" t="s">
+        <v>58</v>
+      </c>
+      <c r="O8" t="s">
+        <v>58</v>
+      </c>
+      <c r="P8" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>58</v>
+      </c>
+      <c r="R8" t="s">
+        <v>58</v>
+      </c>
+      <c r="T8" t="s">
+        <v>58</v>
+      </c>
+      <c r="U8" t="s">
+        <v>58</v>
+      </c>
+      <c r="V8" t="s">
+        <v>58</v>
+      </c>
+      <c r="W8" t="s">
+        <v>56</v>
+      </c>
+      <c r="X8" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AN8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AT8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AU8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AX8" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY8" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA8" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC8" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD8" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" ht="16.5">
+      <c r="A9" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="L9" s="3"/>
+      <c r="M9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="R9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="S9" s="3"/>
+      <c r="T9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="U9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="V9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="W9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="X9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AJ9" s="3"/>
+      <c r="AK9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AM9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AN9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AO9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AP9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AS9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AT9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AU9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AV9" s="3"/>
+      <c r="AW9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AX9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AY9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ9" s="3"/>
+      <c r="BA9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="BB9" s="3"/>
+      <c r="BC9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="BD9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="BE9" s="3"/>
+      <c r="BF9" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" ht="16.5">
+      <c r="A10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M10" t="s">
+        <v>56</v>
+      </c>
+      <c r="N10" t="s">
+        <v>58</v>
+      </c>
+      <c r="O10" t="s">
+        <v>56</v>
+      </c>
+      <c r="P10" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>56</v>
+      </c>
+      <c r="R10" t="s">
+        <v>56</v>
+      </c>
+      <c r="T10" t="s">
+        <v>56</v>
+      </c>
+      <c r="U10" t="s">
+        <v>56</v>
+      </c>
+      <c r="V10" t="s">
+        <v>56</v>
+      </c>
+      <c r="W10" t="s">
+        <v>56</v>
+      </c>
+      <c r="X10" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY10" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA10" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC10" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD10" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" ht="16.5">
+      <c r="A11" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" t="s">
+        <v>56</v>
+      </c>
+      <c r="H11" t="s">
+        <v>56</v>
+      </c>
+      <c r="I11" t="s">
+        <v>56</v>
+      </c>
+      <c r="J11" t="s">
+        <v>56</v>
+      </c>
+      <c r="K11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M11" t="s">
+        <v>56</v>
+      </c>
+      <c r="N11" t="s">
+        <v>58</v>
+      </c>
+      <c r="O11" t="s">
+        <v>56</v>
+      </c>
+      <c r="P11" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>56</v>
+      </c>
+      <c r="R11" t="s">
+        <v>56</v>
+      </c>
+      <c r="T11" t="s">
+        <v>56</v>
+      </c>
+      <c r="U11" t="s">
+        <v>56</v>
+      </c>
+      <c r="V11" t="s">
+        <v>56</v>
+      </c>
+      <c r="W11" t="s">
+        <v>56</v>
+      </c>
+      <c r="X11" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY11" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA11" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC11" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD11" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" ht="16.5">
+      <c r="A12" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="P12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="R12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="W12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AJ12" s="3"/>
+      <c r="AK12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AV12" s="3"/>
+      <c r="AW12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ12" s="3"/>
+      <c r="BA12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BB12" s="3"/>
+      <c r="BC12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BE12" s="3"/>
+      <c r="BF12" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" ht="16.5">
+      <c r="A13" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13" t="s">
+        <v>56</v>
+      </c>
+      <c r="I13" t="s">
+        <v>56</v>
+      </c>
+      <c r="J13" t="s">
+        <v>56</v>
+      </c>
+      <c r="K13" t="s">
+        <v>56</v>
+      </c>
+      <c r="M13" t="s">
+        <v>56</v>
+      </c>
+      <c r="N13" t="s">
+        <v>58</v>
+      </c>
+      <c r="O13" t="s">
+        <v>56</v>
+      </c>
+      <c r="P13" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R13" t="s">
+        <v>56</v>
+      </c>
+      <c r="T13" t="s">
+        <v>56</v>
+      </c>
+      <c r="U13" t="s">
+        <v>56</v>
+      </c>
+      <c r="V13" t="s">
+        <v>56</v>
+      </c>
+      <c r="W13" t="s">
+        <v>56</v>
+      </c>
+      <c r="X13" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX13" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY13" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA13" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC13" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD13" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" ht="16.5">
+      <c r="A14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" t="s">
+        <v>56</v>
+      </c>
+      <c r="I14" t="s">
+        <v>56</v>
+      </c>
+      <c r="J14" t="s">
+        <v>56</v>
+      </c>
+      <c r="K14" t="s">
+        <v>56</v>
+      </c>
+      <c r="M14" t="s">
+        <v>56</v>
+      </c>
+      <c r="N14" t="s">
+        <v>58</v>
+      </c>
+      <c r="O14" t="s">
+        <v>56</v>
+      </c>
+      <c r="P14" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>56</v>
+      </c>
+      <c r="R14" t="s">
+        <v>56</v>
+      </c>
+      <c r="T14" t="s">
+        <v>56</v>
+      </c>
+      <c r="U14" t="s">
+        <v>56</v>
+      </c>
+      <c r="V14" t="s">
+        <v>56</v>
+      </c>
+      <c r="W14" t="s">
+        <v>56</v>
+      </c>
+      <c r="X14" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX14" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY14" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA14" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC14" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD14" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF14" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5">
+      <c r="A15" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" t="s">
+        <v>56</v>
+      </c>
+      <c r="H15" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" t="s">
+        <v>56</v>
+      </c>
+      <c r="J15" t="s">
+        <v>56</v>
+      </c>
+      <c r="K15" t="s">
+        <v>56</v>
+      </c>
+      <c r="M15" t="s">
+        <v>56</v>
+      </c>
+      <c r="N15" t="s">
+        <v>58</v>
+      </c>
+      <c r="O15" t="s">
+        <v>56</v>
+      </c>
+      <c r="P15" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>56</v>
+      </c>
+      <c r="R15" t="s">
+        <v>56</v>
+      </c>
+      <c r="T15" t="s">
+        <v>56</v>
+      </c>
+      <c r="U15" t="s">
+        <v>56</v>
+      </c>
+      <c r="V15" t="s">
+        <v>56</v>
+      </c>
+      <c r="W15" t="s">
+        <v>56</v>
+      </c>
+      <c r="X15" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY15" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA15" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC15" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD15" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" ht="16.5">
+      <c r="A16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" t="s">
+        <v>56</v>
+      </c>
+      <c r="G16" t="s">
+        <v>56</v>
+      </c>
+      <c r="H16" t="s">
+        <v>56</v>
+      </c>
+      <c r="I16" t="s">
+        <v>56</v>
+      </c>
+      <c r="J16" t="s">
+        <v>56</v>
+      </c>
+      <c r="K16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N16" t="s">
+        <v>58</v>
+      </c>
+      <c r="O16" t="s">
+        <v>56</v>
+      </c>
+      <c r="P16" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>56</v>
+      </c>
+      <c r="R16" t="s">
+        <v>56</v>
+      </c>
+      <c r="T16" t="s">
+        <v>56</v>
+      </c>
+      <c r="U16" t="s">
+        <v>56</v>
+      </c>
+      <c r="V16" t="s">
+        <v>56</v>
+      </c>
+      <c r="W16" t="s">
+        <v>56</v>
+      </c>
+      <c r="X16" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI16" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX16" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY16" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA16" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC16" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD16" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" ht="16.5">
+      <c r="A17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" t="s">
+        <v>56</v>
+      </c>
+      <c r="H17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I17" t="s">
+        <v>56</v>
+      </c>
+      <c r="J17" t="s">
+        <v>56</v>
+      </c>
+      <c r="K17" t="s">
+        <v>56</v>
+      </c>
+      <c r="M17" t="s">
+        <v>56</v>
+      </c>
+      <c r="N17" t="s">
+        <v>58</v>
+      </c>
+      <c r="O17" t="s">
+        <v>56</v>
+      </c>
+      <c r="P17" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>56</v>
+      </c>
+      <c r="R17" t="s">
+        <v>56</v>
+      </c>
+      <c r="T17" t="s">
+        <v>56</v>
+      </c>
+      <c r="U17" t="s">
+        <v>56</v>
+      </c>
+      <c r="V17" t="s">
+        <v>56</v>
+      </c>
+      <c r="W17" t="s">
+        <v>56</v>
+      </c>
+      <c r="X17" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI17" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY17" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA17" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC17" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD17" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" ht="16.5">
+      <c r="A18" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G18" t="s">
+        <v>56</v>
+      </c>
+      <c r="H18" t="s">
+        <v>56</v>
+      </c>
+      <c r="I18" t="s">
+        <v>56</v>
+      </c>
+      <c r="J18" t="s">
+        <v>56</v>
+      </c>
+      <c r="K18" t="s">
+        <v>56</v>
+      </c>
+      <c r="M18" t="s">
+        <v>56</v>
+      </c>
+      <c r="N18" t="s">
+        <v>58</v>
+      </c>
+      <c r="O18" t="s">
+        <v>56</v>
+      </c>
+      <c r="P18" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>56</v>
+      </c>
+      <c r="R18" t="s">
+        <v>56</v>
+      </c>
+      <c r="T18" t="s">
+        <v>56</v>
+      </c>
+      <c r="U18" t="s">
+        <v>56</v>
+      </c>
+      <c r="V18" t="s">
+        <v>56</v>
+      </c>
+      <c r="W18" t="s">
+        <v>56</v>
+      </c>
+      <c r="X18" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI18" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY18" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA18" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC18" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD18" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5">
+      <c r="A19" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" t="s">
+        <v>56</v>
+      </c>
+      <c r="I19" t="s">
+        <v>56</v>
+      </c>
+      <c r="J19" t="s">
+        <v>56</v>
+      </c>
+      <c r="K19" t="s">
+        <v>56</v>
+      </c>
+      <c r="M19" t="s">
+        <v>56</v>
+      </c>
+      <c r="N19" t="s">
+        <v>58</v>
+      </c>
+      <c r="O19" t="s">
+        <v>56</v>
+      </c>
+      <c r="P19" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>56</v>
+      </c>
+      <c r="R19" t="s">
+        <v>56</v>
+      </c>
+      <c r="T19" t="s">
+        <v>56</v>
+      </c>
+      <c r="U19" t="s">
+        <v>56</v>
+      </c>
+      <c r="V19" t="s">
+        <v>56</v>
+      </c>
+      <c r="W19" t="s">
+        <v>56</v>
+      </c>
+      <c r="X19" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI19" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX19" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY19" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA19" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC19" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD19" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5">
+      <c r="A20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" t="s">
+        <v>56</v>
+      </c>
+      <c r="H20" t="s">
+        <v>56</v>
+      </c>
+      <c r="I20" t="s">
+        <v>56</v>
+      </c>
+      <c r="J20" t="s">
+        <v>56</v>
+      </c>
+      <c r="K20" t="s">
+        <v>56</v>
+      </c>
+      <c r="M20" t="s">
+        <v>56</v>
+      </c>
+      <c r="N20" t="s">
+        <v>56</v>
+      </c>
+      <c r="O20" t="s">
+        <v>56</v>
+      </c>
+      <c r="P20" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>56</v>
+      </c>
+      <c r="R20" t="s">
+        <v>56</v>
+      </c>
+      <c r="T20" t="s">
+        <v>56</v>
+      </c>
+      <c r="U20" t="s">
+        <v>56</v>
+      </c>
+      <c r="V20" t="s">
+        <v>56</v>
+      </c>
+      <c r="W20" t="s">
+        <v>56</v>
+      </c>
+      <c r="X20" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY20" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA20" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC20" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD20" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" ht="16.5">
+      <c r="A21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" t="s">
+        <v>56</v>
+      </c>
+      <c r="F21" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" t="s">
+        <v>56</v>
+      </c>
+      <c r="H21" t="s">
+        <v>56</v>
+      </c>
+      <c r="I21" t="s">
+        <v>56</v>
+      </c>
+      <c r="J21" t="s">
+        <v>56</v>
+      </c>
+      <c r="K21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M21" t="s">
+        <v>56</v>
+      </c>
+      <c r="N21" t="s">
+        <v>58</v>
+      </c>
+      <c r="O21" t="s">
+        <v>56</v>
+      </c>
+      <c r="P21" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>56</v>
+      </c>
+      <c r="R21" t="s">
+        <v>56</v>
+      </c>
+      <c r="T21" t="s">
+        <v>56</v>
+      </c>
+      <c r="U21" t="s">
+        <v>56</v>
+      </c>
+      <c r="V21" t="s">
+        <v>56</v>
+      </c>
+      <c r="W21" t="s">
+        <v>56</v>
+      </c>
+      <c r="X21" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI21" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AR21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AS21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AU21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX21" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY21" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA21" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC21" t="s">
+        <v>56</v>
+      </c>
+      <c r="BD21" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF21" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="18.75"/>

</xml_diff>